<commit_message>
Preventivas longas: última vez feita e próxima estimada
- Planilha: colunas Última trimestral/semestral/anual e Próxima (calculada), com conferência
- Importação lê as datas e começa o ciclo do plano no mês da próxima (vencida = mês atual)
- preventivas_planos.ultima_execucao, atualizada ao concluir a preventiva (SQL 02)
- Ficha do equipamento mostra última e próxima por plano; edição do plano aceita a data

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KrCh11bbdFjPGwfq6JoneX
</commit_message>
<xml_diff>
--- a/testes/e2e/teste_import.xlsx
+++ b/testes/e2e/teste_import.xlsx
@@ -23,8 +23,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0;\-0.0"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="166" formatCode="DD/MM/YYYY"/>
   </numFmts>
   <fonts count="19">
     <font>
@@ -232,7 +234,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="65">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -426,6 +428,7 @@
     <xf numFmtId="0" fontId="18" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1003,7 +1006,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:R303"/>
+  <dimension ref="A1:T303"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="16" customWidth="1" style="32" min="1" max="1"/>
@@ -1128,6 +1131,16 @@
           <t>Família</t>
         </is>
       </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Última semestral</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>Última anual</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="15" customHeight="1" s="33">
       <c r="A4" s="47" t="inlineStr">
@@ -1434,6 +1447,9 @@
         <f>IF($E8="","",IFERROR(INDEX(Tipos!$B$5:$B$51,MATCH($E8,Tipos!$A$5:$A$51,0)),""))</f>
         <v/>
       </c>
+      <c r="S8" s="65" t="n">
+        <v>46188</v>
+      </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="33">
       <c r="A9" s="50" t="inlineStr">
@@ -1607,6 +1623,11 @@
       <c r="R11" s="49">
         <f>IF($E11="","",IFERROR(INDEX(Tipos!$B$5:$B$51,MATCH($E11,Tipos!$A$5:$A$51,0)),""))</f>
         <v/>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>01/09/2025</t>
+        </is>
       </c>
     </row>
     <row r="12" ht="15" customHeight="1" s="33">

</xml_diff>